<commit_message>
Update UI packaging validation and report standards
</commit_message>
<xml_diff>
--- a/assets/templates/algo_en_full_feature_stateful.xlsx
+++ b/assets/templates/algo_en_full_feature_stateful.xlsx
@@ -1309,7 +1309,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H38"/>
+  <dimension ref="A1:H31"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col width="10" customWidth="1" style="29" min="1" max="1"/>
@@ -2194,16 +2194,16 @@
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>50</v>
+        <v>57</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Learn Command</t>
+          <t>Start Study Light</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Learn Command</t>
+          <t>Start Study Light</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -2213,7 +2213,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Please say the command to learn</t>
+          <t>Okay</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -2223,27 +2223,27 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>A5 FA 00 81 50 00 70 FB</t>
+          <t>A5 FA 00 81 57 00 77 FB</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>A5 FA 00 82 50 00 71 FB</t>
+          <t>A5 FA 00 82 57 00 78 FB</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Learn Wake Word</t>
+          <t>Stop Study Light</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Learn Wake Word</t>
+          <t>Stop Study Light</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -2253,7 +2253,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Please say the wake word to learn</t>
+          <t>Okay</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -2263,27 +2263,27 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>A5 FA 00 81 51 00 71 FB</t>
+          <t>A5 FA 00 81 58 00 78 FB</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>A5 FA 00 82 51 00 72 FB</t>
+          <t>A5 FA 00 82 58 00 79 FB</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>52</v>
+        <v>30</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Delete Command</t>
+          <t>Query Device Status</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Delete Command</t>
+          <t>Query Device Status</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -2293,380 +2293,100 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Please say the command to delete</t>
+          <t>Current status is normal</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>主</t>
+          <t>被</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>A5 FA 00 81 52 00 72 FB</t>
+          <t>A5 FA 00 81 30 00 50 FB</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>A5 FA 00 82 52 00 73 FB</t>
+          <t>A5 FA 00 82 30 00 51 FB</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>53</v>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>Delete Wake Word</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>Delete Wake Word</t>
-        </is>
+        <v>31</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>命令词</t>
+          <t>播报语</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Please say the wake word to delete</t>
+          <t>Passive status is normal</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>主</t>
+          <t>被</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>A5 FA 00 81 53 00 73 FB</t>
+          <t>A5 FA 00 81 31 00 51 FB</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>A5 FA 00 82 53 00 74 FB</t>
+          <t>A5 FA 00 82 31 00 52 FB</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>54</v>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>Delete All Commands</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>Delete All Commands</t>
-        </is>
+        <v>32</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>命令词</t>
+          <t>播报语</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>All commands deleted</t>
+          <t>Protocol broadcast triggered</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>主</t>
+          <t>被</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>A5 FA 00 81 54 00 74 FB</t>
+          <t>A5 FA 00 81 32 00 52 FB</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>A5 FA 00 82 54 00 75 FB</t>
+          <t>A5 FA 00 82 32 00 53 FB</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>55</v>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>Exit Learning</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>Exit Learning</t>
-        </is>
+        <v>33</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>命令词</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>Learning exited</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>主</t>
+          <t>心跳协议</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>A5 FA 00 81 55 00 75 FB</t>
+          <t>A5 FA 00 81 33 00 53 FB</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
-        <is>
-          <t>A5 FA 00 82 55 00 76 FB</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="n">
-        <v>56</v>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>Exit Deletion</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>Exit Deletion</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>命令词</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>Deletion exited</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>主</t>
-        </is>
-      </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>A5 FA 00 81 56 00 76 FB</t>
-        </is>
-      </c>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>A5 FA 00 82 56 00 77 FB</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="n">
-        <v>57</v>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>Start Study Light</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>Start Study Light</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>命令词</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>Okay</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>主</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>A5 FA 00 81 57 00 77 FB</t>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>A5 FA 00 82 57 00 78 FB</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="n">
-        <v>58</v>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>Stop Study Light</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>Stop Study Light</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>命令词</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>Okay</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>主</t>
-        </is>
-      </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>A5 FA 00 81 58 00 78 FB</t>
-        </is>
-      </c>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>A5 FA 00 82 58 00 79 FB</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="n">
-        <v>30</v>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>Query Device Status</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>Query Device Status</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>命令词</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>Current status is normal</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>被</t>
-        </is>
-      </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>A5 FA 00 81 30 00 50 FB</t>
-        </is>
-      </c>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>A5 FA 00 82 30 00 51 FB</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="n">
-        <v>31</v>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>播报语</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>Passive status is normal</t>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>被</t>
-        </is>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>A5 FA 00 81 31 00 51 FB</t>
-        </is>
-      </c>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>A5 FA 00 82 31 00 52 FB</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="n">
-        <v>32</v>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>播报语</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>Protocol broadcast triggered</t>
-        </is>
-      </c>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>被</t>
-        </is>
-      </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>A5 FA 00 81 32 00 52 FB</t>
-        </is>
-      </c>
-      <c r="H37" t="inlineStr">
-        <is>
-          <t>A5 FA 00 82 32 00 53 FB</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="n">
-        <v>33</v>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>心跳协议</t>
-        </is>
-      </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>A5 FA 00 81 33 00 53 FB</t>
-        </is>
-      </c>
-      <c r="H38" t="inlineStr">
         <is>
           <t>A5 FA 00 82 33 00 54 FB</t>
         </is>

</xml_diff>